<commit_message>
Complete Module Certification Sprint
</commit_message>
<xml_diff>
--- a/BandConnect_Data_Dictionary.xlsx
+++ b/BandConnect_Data_Dictionary.xlsx
@@ -19825,7 +19825,7 @@
       </c>
       <c r="C40" s="32" t="inlineStr">
         <is>
-          <t>Groups permissions for admin categorisation display.</t>
+          <t>Groups related permission tokens for admin UI categorisation.</t>
         </is>
       </c>
       <c r="D40" s="29" t="n"/>
@@ -20818,7 +20818,7 @@
       </c>
       <c r="F28" s="32" t="inlineStr">
         <is>
-          <t>Groups permissions for admin categorisation display.</t>
+          <t>Groups related permission tokens for admin UI categorisation.</t>
         </is>
       </c>
       <c r="G28" s="29" t="n"/>
@@ -21074,7 +21074,7 @@
       </c>
       <c r="C42" s="32" t="inlineStr">
         <is>
-          <t>Groups permissions for admin categorisation display.</t>
+          <t>Groups related permission tokens for admin UI categorisation.</t>
         </is>
       </c>
       <c r="D42" s="29" t="n"/>
@@ -39413,7 +39413,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Groups permissions for admin categorisation display.</t>
+          <t>Groups related permission tokens for admin UI categorisation.</t>
         </is>
       </c>
     </row>
@@ -42215,7 +42215,7 @@
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>Groups permissions for admin categorisation display.</t>
+          <t>Groups related permission tokens for admin UI categorisation.</t>
         </is>
       </c>
     </row>

</xml_diff>